<commit_message>
Cap nhat bai 7 test data phan vung tuong duong
</commit_message>
<xml_diff>
--- a/Buoi2_NguyenHoTruongTam_11CNPM2/Lab2_NguyenHoTruongTam_11CNPM2.xlsx
+++ b/Buoi2_NguyenHoTruongTam_11CNPM2/Lab2_NguyenHoTruongTam_11CNPM2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\A.monhoc\software-testing\Buoi2_NguyenHoTruongTam_11CNPM2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDCFD47A-EFA4-46CC-904F-D9EA46A1F578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12D5E59B-0C20-4CA8-95EB-856EBBCF8C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bai1_LaiSuat" sheetId="2" r:id="rId1"/>
@@ -707,27 +707,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="163"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="163"/>
     </font>
     <font>
       <b/>
@@ -754,17 +740,12 @@
       <scheme val="major"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8F0FE"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -800,29 +781,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1130,235 +1100,235 @@
   <dimension ref="A1:D39"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10" style="7" customWidth="1"/>
-    <col min="2" max="2" width="16" style="7" customWidth="1"/>
-    <col min="3" max="3" width="12" style="7" customWidth="1"/>
-    <col min="4" max="4" width="48" style="7" customWidth="1"/>
-    <col min="5" max="16384" width="8.796875" style="7"/>
+    <col min="1" max="1" width="10" style="2" customWidth="1"/>
+    <col min="2" max="2" width="16" style="2" customWidth="1"/>
+    <col min="3" max="3" width="12" style="2" customWidth="1"/>
+    <col min="4" max="4" width="48" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="8.796875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="10" t="s">
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="10" t="s">
+      <c r="B6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="10" t="s">
+      <c r="B7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="5" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="11" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="5">
         <v>50</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="5">
         <v>100</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="5">
         <v>999</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="5">
         <v>1000</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="5" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="5">
         <v>0</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="5">
         <v>-10</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="5" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="5" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10" t="s">
+      <c r="B20" s="5"/>
+      <c r="C20" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="5" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1374,13 +1344,13 @@
     <row r="30" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1391,228 +1361,228 @@
   <dimension ref="A1:D49"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="73.69921875" style="7" customWidth="1"/>
-    <col min="2" max="2" width="20" style="7" customWidth="1"/>
-    <col min="3" max="3" width="51.796875" style="7" customWidth="1"/>
-    <col min="4" max="4" width="50" style="7" customWidth="1"/>
-    <col min="5" max="16384" width="8.796875" style="7"/>
+    <col min="1" max="1" width="73.69921875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20" style="2" customWidth="1"/>
+    <col min="3" max="3" width="51.796875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="50" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="8.796875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="1" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="21.6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="3"/>
     </row>
     <row r="4" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
+      <c r="A4" s="3"/>
     </row>
     <row r="5" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="10" t="s">
+      <c r="B8" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="5" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="5" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="5" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="5" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="5" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="4" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="5" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="5" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="5" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="5" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10" t="s">
+      <c r="B22" s="5"/>
+      <c r="C22" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="5" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1626,23 +1596,23 @@
     <row r="30" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1653,377 +1623,377 @@
   <dimension ref="A1:E69"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="49.69921875" style="7" customWidth="1"/>
-    <col min="2" max="2" width="18" style="7" customWidth="1"/>
-    <col min="3" max="3" width="34.8984375" style="7" customWidth="1"/>
-    <col min="4" max="4" width="37.59765625" style="7" customWidth="1"/>
-    <col min="5" max="5" width="36" style="7" customWidth="1"/>
-    <col min="6" max="16384" width="8.796875" style="7"/>
+    <col min="1" max="1" width="49.69921875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="18" style="2" customWidth="1"/>
+    <col min="3" max="3" width="34.8984375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="37.59765625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="36" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="8.796875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="1" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="3" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="3" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="6" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="5" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="5" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="5" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="6" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="10" t="s">
+      <c r="B14" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="5" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="B15" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="5" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C16" s="10" t="s">
+      <c r="B16" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="5" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="B17" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C17" s="10" t="s">
+      <c r="B17" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="5" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="5" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="5" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="4" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="D22" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="5" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="5" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
+      <c r="A25" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="5" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="5" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="5" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" s="5" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="10" t="s">
+      <c r="A29" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D29" s="5" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
+      <c r="A30" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10" t="s">
+      <c r="B30" s="5"/>
+      <c r="C30" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" s="5" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="52" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="53" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="54" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="55" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="57" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="60" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="61" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="67" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="68" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="69" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2034,390 +2004,390 @@
   <dimension ref="A1:D79"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="53.19921875" style="7" customWidth="1"/>
-    <col min="2" max="2" width="18" style="7" customWidth="1"/>
-    <col min="3" max="3" width="44.8984375" style="7" customWidth="1"/>
-    <col min="4" max="4" width="55" style="7" customWidth="1"/>
-    <col min="5" max="16384" width="8.796875" style="7"/>
+    <col min="1" max="1" width="53.19921875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="18" style="2" customWidth="1"/>
+    <col min="3" max="3" width="44.8984375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="55" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="8.796875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="3"/>
     </row>
     <row r="4" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="6" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="10" t="s">
+      <c r="B7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="5" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="10" t="s">
+      <c r="B8" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="5" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="10" t="s">
+      <c r="B9" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="5" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="5" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="5" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="5" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="5" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="5" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="4" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="5">
         <v>40</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="5" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="5">
         <v>99</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="5" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="5">
         <v>100</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="5" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="5">
         <v>140</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="5" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="5">
         <v>141</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="5" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="10">
+      <c r="B23" s="5">
         <v>200</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="5" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="5">
         <v>20</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="5" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
+      <c r="A25" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="10">
+      <c r="B25" s="5">
         <v>201</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="5" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="5">
         <v>-5</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="5" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="5">
         <v>160.5</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="5" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" s="5" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="10" t="s">
+      <c r="A29" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10" t="s">
+      <c r="B29" s="5"/>
+      <c r="C29" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D29" s="5" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="70" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="72" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="73" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="75" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="76" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="77" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="78" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="79" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="52" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="53" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="54" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="55" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="57" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="60" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="61" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="67" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="68" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="69" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="70" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="71" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="72" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="73" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="74" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="75" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="76" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="77" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="78" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="79" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2428,267 +2398,267 @@
   <dimension ref="A1:D69"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10" style="7" customWidth="1"/>
-    <col min="2" max="2" width="14" style="7" customWidth="1"/>
-    <col min="3" max="3" width="12" style="7" customWidth="1"/>
-    <col min="4" max="4" width="58" style="7" customWidth="1"/>
-    <col min="5" max="16384" width="8.796875" style="7"/>
+    <col min="1" max="1" width="10" style="2" customWidth="1"/>
+    <col min="2" max="2" width="14" style="2" customWidth="1"/>
+    <col min="3" max="3" width="12" style="2" customWidth="1"/>
+    <col min="4" max="4" width="58" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="8.796875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="1" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="3"/>
     </row>
     <row r="4" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="6" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="10" t="s">
+      <c r="B7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="5" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="10" t="s">
+      <c r="B8" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="5" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="5" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="5" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="5" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="5" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="4" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="5">
         <v>20</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="5" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="5">
         <v>25</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="5" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="5">
         <v>26</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="5" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="5">
         <v>30</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="5" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="5">
         <v>19</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="5" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="5">
         <v>31</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="5" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="5">
         <v>24.5</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="5" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="5" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10" t="s">
+      <c r="B24" s="5"/>
+      <c r="C24" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="5" t="s">
         <v>108</v>
       </c>
     </row>
@@ -2700,43 +2670,43 @@
     <row r="30" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="52" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="53" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="54" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="55" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="57" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="60" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="61" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="67" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="68" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="69" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2747,291 +2717,291 @@
   <dimension ref="A1:D59"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10" style="7" customWidth="1"/>
-    <col min="2" max="2" width="14" style="7" customWidth="1"/>
-    <col min="3" max="3" width="12" style="7" customWidth="1"/>
-    <col min="4" max="4" width="60" style="7" customWidth="1"/>
-    <col min="5" max="16384" width="8.796875" style="7"/>
+    <col min="1" max="1" width="10" style="2" customWidth="1"/>
+    <col min="2" max="2" width="14" style="2" customWidth="1"/>
+    <col min="3" max="3" width="12" style="2" customWidth="1"/>
+    <col min="4" max="4" width="60" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="8.796875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="1" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="4" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="6" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="5" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="10" t="s">
+      <c r="B6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="5" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="5" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="10" t="s">
+      <c r="B8" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="5" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="5" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="5" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="5" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="4" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="5">
         <v>1</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="5">
         <v>10</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="5">
         <v>20</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="5">
         <v>30</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="5">
         <v>0</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="5" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="5">
         <v>15</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="5" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="5">
         <v>31</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="5" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="5">
         <v>7.2</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="5" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="5" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10" t="s">
+      <c r="B24" s="5"/>
+      <c r="C24" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="5" t="s">
         <v>69</v>
       </c>
     </row>
@@ -3043,33 +3013,33 @@
     <row r="30" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" s="7" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="52" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="53" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="54" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="55" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="57" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3080,383 +3050,384 @@
   <dimension ref="A1:I119"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="8" customWidth="1"/>
-    <col min="4" max="8" width="7" customWidth="1"/>
-    <col min="9" max="9" width="40" customWidth="1"/>
+    <col min="1" max="1" width="10" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24" style="2" customWidth="1"/>
+    <col min="3" max="3" width="8" style="2" customWidth="1"/>
+    <col min="4" max="8" width="7" style="2" customWidth="1"/>
+    <col min="9" max="9" width="40" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="8.796875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="3" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="3" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="4" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="6" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="4" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G14" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="H14" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="I14" s="6" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="5">
         <v>8</v>
       </c>
-      <c r="E15" s="4">
-        <v>7</v>
-      </c>
-      <c r="F15" s="4">
+      <c r="E15" s="5">
+        <v>7</v>
+      </c>
+      <c r="F15" s="5">
         <v>6</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="5">
         <v>5</v>
       </c>
-      <c r="H15" s="4">
+      <c r="H15" s="5">
         <v>9</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="I15" s="5" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="5">
         <v>4</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="5">
         <v>5</v>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="5">
         <v>6</v>
       </c>
-      <c r="G16" s="4">
+      <c r="G16" s="5">
         <v>5</v>
       </c>
-      <c r="H16" s="4">
+      <c r="H16" s="5">
         <v>5</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="5" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="5">
         <v>0</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="5">
         <v>0</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="5">
         <v>0</v>
       </c>
-      <c r="G17" s="4">
+      <c r="G17" s="5">
         <v>0</v>
       </c>
-      <c r="H17" s="4">
+      <c r="H17" s="5">
         <v>0</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="I17" s="5" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="5">
         <v>10</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="5">
         <v>10</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="5">
         <v>10</v>
       </c>
-      <c r="G18" s="4">
+      <c r="G18" s="5">
         <v>10</v>
       </c>
-      <c r="H18" s="4">
+      <c r="H18" s="5">
         <v>10</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="I18" s="5" t="s">
         <v>207</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="5">
         <v>8</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="5">
         <v>8</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="5">
         <v>8</v>
       </c>
-      <c r="G19" s="4">
+      <c r="G19" s="5">
         <v>8</v>
       </c>
-      <c r="H19" s="4">
+      <c r="H19" s="5">
         <v>8</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="I19" s="5" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="D20" s="4">
-        <v>7</v>
-      </c>
-      <c r="E20" s="4">
-        <v>7</v>
-      </c>
-      <c r="F20" s="4">
-        <v>7</v>
-      </c>
-      <c r="G20" s="4">
-        <v>7</v>
-      </c>
-      <c r="H20" s="4">
-        <v>7</v>
-      </c>
-      <c r="I20" s="4" t="s">
+      <c r="D20" s="5">
+        <v>7</v>
+      </c>
+      <c r="E20" s="5">
+        <v>7</v>
+      </c>
+      <c r="F20" s="5">
+        <v>7</v>
+      </c>
+      <c r="G20" s="5">
+        <v>7</v>
+      </c>
+      <c r="H20" s="5">
+        <v>7</v>
+      </c>
+      <c r="I20" s="5" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="5">
         <v>-1</v>
       </c>
-      <c r="E21" s="4">
-        <v>7</v>
-      </c>
-      <c r="F21" s="4">
-        <v>7</v>
-      </c>
-      <c r="G21" s="4">
-        <v>7</v>
-      </c>
-      <c r="H21" s="4">
-        <v>7</v>
-      </c>
-      <c r="I21" s="4" t="s">
+      <c r="E21" s="5">
+        <v>7</v>
+      </c>
+      <c r="F21" s="5">
+        <v>7</v>
+      </c>
+      <c r="G21" s="5">
+        <v>7</v>
+      </c>
+      <c r="H21" s="5">
+        <v>7</v>
+      </c>
+      <c r="I21" s="5" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D22" s="5">
         <v>11</v>
       </c>
-      <c r="E22" s="4">
-        <v>7</v>
-      </c>
-      <c r="F22" s="4">
-        <v>7</v>
-      </c>
-      <c r="G22" s="4">
-        <v>7</v>
-      </c>
-      <c r="H22" s="4">
-        <v>7</v>
-      </c>
-      <c r="I22" s="4" t="s">
+      <c r="E22" s="5">
+        <v>7</v>
+      </c>
+      <c r="F22" s="5">
+        <v>7</v>
+      </c>
+      <c r="G22" s="5">
+        <v>7</v>
+      </c>
+      <c r="H22" s="5">
+        <v>7</v>
+      </c>
+      <c r="I22" s="5" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="E23" s="4">
-        <v>7</v>
-      </c>
-      <c r="F23" s="4">
-        <v>7</v>
-      </c>
-      <c r="G23" s="4">
-        <v>7</v>
-      </c>
-      <c r="H23" s="4">
-        <v>7</v>
-      </c>
-      <c r="I23" s="4" t="s">
+      <c r="E23" s="5">
+        <v>7</v>
+      </c>
+      <c r="F23" s="5">
+        <v>7</v>
+      </c>
+      <c r="G23" s="5">
+        <v>7</v>
+      </c>
+      <c r="H23" s="5">
+        <v>7</v>
+      </c>
+      <c r="I23" s="5" t="s">
         <v>224</v>
       </c>
     </row>
@@ -3469,93 +3440,93 @@
     <row r="30" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="70" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="72" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="73" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="75" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="76" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="77" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="78" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="79" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="80" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="81" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="82" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="83" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="84" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="85" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="86" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="87" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="88" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="89" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="90" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="91" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="92" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="93" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="94" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="95" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="96" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="97" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="98" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="99" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="100" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="101" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="102" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="103" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="104" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="105" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="106" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="107" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="108" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="109" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="110" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="111" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="112" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="113" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="114" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="115" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="116" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="117" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="118" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="119" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="52" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="53" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="54" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="55" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="57" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="60" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="61" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="67" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="68" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="69" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="70" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="71" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="72" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="73" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="74" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="75" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="76" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="77" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="78" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="79" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="80" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="81" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="82" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="83" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="84" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="85" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="86" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="87" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="88" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="89" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="90" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="91" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="92" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="93" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="94" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="95" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="96" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="97" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="98" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="99" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="100" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="101" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="102" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="103" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="104" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="105" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="106" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="107" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="108" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="109" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="110" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="111" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="112" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="113" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="114" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="115" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="116" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="117" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="118" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="119" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>